<commit_message>
Update berita 2026-08-05 05:28 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-03.xlsx
+++ b/data/berita_2026-08-03.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -778,8 +778,312 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Uji Coba Tabung CNG 3 Kg Masuk Tahap Akhir</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 22:58:12 +0700</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Menteri ESDM Bahlil Lahadalia menyampaikan tabung Compressed Natural Gas (CNG) 3 kilogram (kg) sebagai pengganti LPG 3 kg memasuki pengujian tahap akhir.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8603105/uji-coba-tabung-cng-3-kg-masuk-tahap-akhir</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/20/cadangan-gas-raksasa-ditemukan-di-kaltim-pemerintah-genjot-energi-nasional-1776674766178_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dapat Margin Fee 7%, Bulog Targetkan Untung Rp 1,14 Triliun</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 22:32:25 +0700</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pemerintah menetapkan margin fee untuk Perum Bulog sebesar 7%</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/industri/d-8603085/dapat-margin-fee-7-bulog-targetkan-untung-rp-1-14-triliun</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/02/22/f0bc228f-67f0-4a85-b1de-c8b83e0fc898_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pemerintah Kejar Rasio Wirausaha 8 Persen pada 2045</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 22:00:05 +0700</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>UMKM makanan siap saji menjadi salah satu penggerak kewirausahaan nasional. Sejalan dengan pemerintah menargetkan rasio wirausaha mencapai 8 persen pada 2045.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8602134/pemerintah-kejar-rasio-wirausaha-8-persen-pada-2045</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/03/pemerintah-kejar-rasio-wirausaha-8-persen-pada-2045-1785739243678.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BULOG Dapat Dukungan Finansial Penuh dari Pemerintah untuk Swasembada</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 21:54:32 +0700</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Perum BULOG mengapresiasi dukungan pemerintah dalam memperkuat perannya sebagai operator pangan nasional.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/ekonomi-bisnis/d-8603050/bulog-dapat-dukungan-finansial-penuh-dari-pemerintah-untuk-swasembada</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/03/direktur-utama-dirut-perum-bulog-letnan-jenderal-tni-purn-ahmad-rizal-ramdhani-1785768755808.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bulog Jamin MBG Tak Pakai Beras SPHP dan Minyakita</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 21:45:27 +0700</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Perum Bulog memastikan bahan pangan untuk program makan bergizi gratis (MBG) merupakan produk premium, bukan beras SPHP maupun Minyakita.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8603041/bulog-jamin-mbg-tak-pakai-beras-sphp-dan-minyakita</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/12/29/dirut-bulog-ahmad-rizal-ramdhani-1767018144863_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tawarkan Pasok Beras Berkualitas, Thailand Mau Impor Pupuk RI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 21:12:37 +0700</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Perdana Menteri (PM) Thailand Anutin Charnvirakul berharap Indonesia dan Thailand semakin mempererat kerja sama di sektor pangan.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8603009/tawarkan-pasok-beras-berkualitas-thailand-mau-impor-pupuk-ri</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/03/prabowo-terima-kunjungan-pm-thailand-kerja-sama-bilateral-makin-diperkuat-1785753891165_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BNI Hadirkan Ekosistem Keuangan Digital bagi Mahasiswa RI di Hong Kong</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 20:53:27 +0700</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BNI perluas layanan keuangan digital untuk mahasiswa Indonesia di Hong Kong, termasuk pembukaan rekening dan kartu debit multicurrency.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8602989/bni-hadirkan-ekosistem-keuangan-digital-bagi-mahasiswa-ri-di-hong-kong</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/03/bni-1785765055910_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bicara Investasi, PM Thailand Ungkap Bangkok Bank Caplok Bank Permata</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 20:08:33 +0700</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto menerima kunjungan Perdana Menteri (PM) Thailand Anutin Charnvirakul di Istana Kepresidenan.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8602936/bicara-investasi-pm-thailand-ungkap-bangkok-bank-caplok-bank-permata</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/03/prabowo-terima-kunjungan-pm-thailand-kerja-sama-bilateral-makin-diperkuat-1785753891099_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H9"/>
+  <autoFilter ref="A1:H17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 12:55 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-03.xlsx
+++ b/data/berita_2026-08-03.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,10 +419,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
@@ -3112,8 +3112,55 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Malaysia Selidiki Pilot Penyelundup Narkoba ke RI Bisa Lolos di KLIA</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 23:43:03 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Pilot Malaysia ditangkap di Indonesia karena menyelundupkan 26 kg narkoba. Investigasi mendalam dilakukan terkait kelolosan pemeriksaan di bandara.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260803231914-106-1388224/malaysia-selidiki-pilot-penyelundup-narkoba-ke-ri-bisa-lolos-di-klia</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/04/pilot-maskapai-asing-asal-malaysia-mohd-saufi-bin-othman-mso-ditangkap-tim-gabungan-bareskrim-polri-dan-bea-cukai-bandara-soek-1785826709010_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I57"/>
+  <autoFilter ref="A1:I58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>